<commit_message>
data: corrige tildes y signos de apertura en los textos visibles
Solo cambian textos mostrados al usuario; ids, valores de opciones, condiciones, URLs, siglas y codigos quedan iguales. El motor da el mismo resultado (6/6); en resultados-motor.json solo cambian los mensajes de alerta.
</commit_message>
<xml_diff>
--- a/data/ruta-obra.xlsx
+++ b/data/ruta-obra.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Informacion referencial. No es asesoria legal. Montos y plazos deben confirmarse en el TUPA vigente de cada entidad antes de presentar un tramite.</t>
+          <t>Información referencial. No es asesoría legal. Montos y plazos deben confirmarse en el TUPA vigente de cada entidad antes de presentar un trámite.</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dato leido en la fuente oficial citada.</t>
+          <t>Dato leído en la fuente oficial citada.</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dato oficial de una version anterior del TUPA o norma; confirmar vigencia.</t>
+          <t>Dato oficial de una versión anterior del TUPA o norma; confirmar vigencia.</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Como esta la propiedad del terreno hoy?</t>
+          <t>¿Cómo está la propiedad del terreno hoy?</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "inscrito", "etiqueta": "Inscrita en SUNARP a mi nombre"}, {"valor": "compraventa_no_inscrita", "etiqueta": "Tengo contrato o minuta de compraventa, sin inscribir"}, {"valor": "posesion_estatal", "etiqueta": "Posesion en terreno del Estado, sin titulo"}, {"valor": "posesion_privada", "etiqueta": "Posesion en terreno privado por mas de 10 anos, sin titulo"}, {"valor": "herencia", "etiqueta": "Heredada, a nombre de un familiar fallecido"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "inscrito", "etiqueta": "Inscrita en SUNARP a mi nombre"}, {"valor": "compraventa_no_inscrita", "etiqueta": "Tengo contrato o minuta de compraventa, sin inscribir"}, {"valor": "posesion_estatal", "etiqueta": "Posesión en terreno del Estado, sin título"}, {"valor": "posesion_privada", "etiqueta": "Posesión en terreno privado por más de 10 años, sin título"}, {"valor": "herencia", "etiqueta": "Heredada, a nombre de un familiar fallecido"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
@@ -687,7 +687,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>El predio tiene partida registral propia (no es parte de un lote mayor)?</t>
+          <t>¿El predio tiene partida registral propia (no es parte de un lote mayor)?</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No, es parte de un lote mayor"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No, es parte de un lote mayor"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
@@ -715,7 +715,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Ya hay algo construido en el terreno?</t>
+          <t>¿Ya hay algo construido en el terreno?</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "no", "etiqueta": "No, terreno libre"}, {"valor": "si_declarada", "etiqueta": "Si, y esta declarada en SUNARP"}, {"valor": "si_sin_declarar", "etiqueta": "Si, pero sin licencia o sin declarar"}]</t>
+          <t>[{"valor": "no", "etiqueta": "No, terreno libre"}, {"valor": "si_declarada", "etiqueta": "Sí, y está declarada en SUNARP"}, {"valor": "si_sin_declarar", "etiqueta": "Sí, pero sin licencia o sin declarar"}]</t>
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Cuando se termino lo construido sin licencia?</t>
+          <t>¿Cuándo se terminó lo construido sin licencia?</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "hasta_2016", "etiqueta": "Hasta el 31-12-2016"}, {"valor": "2017_sep2018", "etiqueta": "Entre el 01-01-2017 y el 17-09-2018"}, {"valor": "post_sep2018", "etiqueta": "Despues del 17-09-2018"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "hasta_2016", "etiqueta": "Hasta el 31-12-2016"}, {"valor": "2017_sep2018", "etiqueta": "Entre el 01-01-2017 y el 17-09-2018"}, {"valor": "post_sep2018", "etiqueta": "Después del 17-09-2018"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>En que distrito esta el predio?</t>
+          <t>¿En qué distrito está el predio?</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>El predio esta en alguna de estas zonas?</t>
+          <t>¿El predio está en alguna de estas zonas?</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "pantanos_villa", "etiqueta": "Cerca de los Pantanos de Villa"}, {"valor": "anp", "etiqueta": "Area natural protegida o su zona de amortiguamiento"}, {"valor": "monumental", "etiqueta": "Zona monumental o inmueble historico"}, {"valor": "ninguna", "etiqueta": "Ninguna"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "pantanos_villa", "etiqueta": "Cerca de los Pantanos de Villa"}, {"valor": "anp", "etiqueta": "Área natural protegida o su zona de amortiguamiento"}, {"valor": "monumental", "etiqueta": "Zona monumental o inmueble histórico"}, {"valor": "ninguna", "etiqueta": "Ninguna"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F7" s="6" t="n"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Que quieres hacer?</t>
+          <t>¿Qué quieres hacer?</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "obra_nueva", "etiqueta": "Construir desde cero"}, {"valor": "ampliacion", "etiqueta": "Ampliar (mas pisos o mas area)"}, {"valor": "remodelacion", "etiqueta": "Remodelar"}, {"valor": "demolicion", "etiqueta": "Demoler"}, {"valor": "cerco", "etiqueta": "Solo cerco perimetrico"}]</t>
+          <t>[{"valor": "obra_nueva", "etiqueta": "Construir desde cero"}, {"valor": "ampliacion", "etiqueta": "Ampliar (más pisos o más área)"}, {"valor": "remodelacion", "etiqueta": "Remodelar"}, {"valor": "demolicion", "etiqueta": "Demoler"}, {"valor": "cerco", "etiqueta": "Solo cerco perimétrico"}]</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
@@ -859,7 +859,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Para que uso?</t>
+          <t>¿Para qué uso?</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "vivienda_unifamiliar", "etiqueta": "Vivienda de una familia"}, {"valor": "vivienda_multifamiliar", "etiqueta": "Vivienda de varias familias / departamentos"}, {"valor": "comercio", "etiqueta": "Comercio u oficinas"}, {"valor": "mixto", "etiqueta": "Vivienda + comercio"}, {"valor": "industria", "etiqueta": "Industria"}, {"valor": "educacion_salud_hospedaje", "etiqueta": "Educacion, salud u hospedaje"}]</t>
+          <t>[{"valor": "vivienda_unifamiliar", "etiqueta": "Vivienda de una familia"}, {"valor": "vivienda_multifamiliar", "etiqueta": "Vivienda de varias familias / departamentos"}, {"valor": "comercio", "etiqueta": "Comercio u oficinas"}, {"valor": "mixto", "etiqueta": "Vivienda + comercio"}, {"valor": "industria", "etiqueta": "Industria"}, {"valor": "educacion_salud_hospedaje", "etiqueta": "Educación, salud u hospedaje"}]</t>
         </is>
       </c>
       <c r="F9" s="6" t="n"/>
@@ -887,7 +887,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Cuantos pisos tendra en total?</t>
+          <t>¿Cuántos pisos tendrá en total?</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Area techada total al terminar (m2)</t>
+          <t>Área techada total al terminar (m²)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>La obra modifica la estructura (columnas, vigas, losas)?</t>
+          <t>¿La obra modifica la estructura (columnas, vigas, losas)?</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Habra sotano o excavacion de mas de 2 m?</t>
+          <t>¿Habrá sótano o excavación de más de 2 m?</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}]</t>
         </is>
       </c>
       <c r="F13" s="6" t="n"/>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Como piensas financiarla?</t>
+          <t>¿Cómo piensas financiarla?</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "techo_propio", "etiqueta": "Bono Techo Propio"}, {"valor": "credito", "etiqueta": "Credito hipotecario / MiVivienda"}, {"valor": "propio", "etiqueta": "Recursos propios"}]</t>
+          <t>[{"valor": "techo_propio", "etiqueta": "Bono Techo Propio"}, {"valor": "credito", "etiqueta": "Crédito hipotecario / MiVivienda"}, {"valor": "propio", "etiqueta": "Recursos propios"}]</t>
         </is>
       </c>
       <c r="F15" s="6" t="n"/>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Contrataras maestro de obra y obreros?</t>
+          <t>¿Contratarás maestro de obra y obreros?</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}]</t>
         </is>
       </c>
       <c r="F16" s="6" t="n"/>
@@ -2067,7 +2067,7 @@
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Segun envergadura; confirmar con la municipalidad</t>
+          <t>Según envergadura; confirmar con la municipalidad</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>Lo construido despues del 17-09-2018 solo se regulariza si tu distrito tiene una ordenanza de beneficio vigente. Sin ella hay riesgo de multa o demolicion.</t>
+          <t>Lo construido después del 17-09-2018 solo se regulariza si tu distrito tiene una ordenanza de beneficio vigente. Sin ella hay riesgo de multa o demolición.</t>
         </is>
       </c>
       <c r="M40" s="6" t="n"/>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>Necesitas opinion de PROHVILLA antes de la licencia. Suele ser la etapa mas larga: iniciala en paralelo con los documentos previos. Alturas de 2 a 4 pisos y area libre de 30% a 60% segun zona.</t>
+          <t>Necesitas opinión de PROHVILLA antes de la licencia. Suele ser la etapa más larga: iníciala en paralelo con los documentos previos. Alturas de 2 a 4 pisos y área libre de 30% a 60% según zona.</t>
         </is>
       </c>
       <c r="M41" s="6" t="n"/>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>Pide primero el certificado de parametros: indica si el predio esta en zona especial.</t>
+          <t>Pide primero el certificado de parámetros: indica si el predio está en zona especial.</t>
         </is>
       </c>
       <c r="M42" s="6" t="n"/>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="L43" s="6" t="inlineStr">
         <is>
-          <t>Excavaciones de mas de 2 m requieren plano de sostenimiento.</t>
+          <t>Excavaciones de más de 2 m requieren plano de sostenimiento.</t>
         </is>
       </c>
       <c r="M43" s="6" t="n"/>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
-          <t>Tu distrito aun no tiene tasas cargadas: la ruta es valida (norma nacional), pero montos y canal deben confirmarse en su TUPA.</t>
+          <t>Tu distrito aún no tiene tasas cargadas: la ruta es válida (norma nacional), pero montos y canal deben confirmarse en su TUPA.</t>
         </is>
       </c>
       <c r="M45" s="6" t="n"/>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>La copia literal vence: la licencia exige maximo 30 dias de antiguedad.</t>
+          <t>La copia literal vence: la licencia exige máximo 30 días de antigüedad.</t>
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>El certificado de parametros vence (36 meses).</t>
+          <t>El certificado de parámetros vence (36 meses).</t>
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>La licencia vence (36 meses). Pide la prorroga de 12 meses ANTES del vencimiento.</t>
+          <t>La licencia vence (36 meses). Pide la prórroga de 12 meses ANTES del vencimiento.</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Tienes 5 dias habiles para subsanar observaciones (prorrogables 5 mas en algunos distritos).</t>
+          <t>Tienes 5 días hábiles para subsanar observaciones (prorrogables 5 más en algunos distritos).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Ley de Regulacion de Habilitaciones Urbanas y de Edificaciones</t>
+          <t>Ley de Regulación de Habilitaciones Urbanas y de Edificaciones</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Modifica la Ley 29090 (regularizacion art. 30)</t>
+          <t>Modifica la Ley 29090 (regularización art. 30)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Reglamento de Licencias de Habilitacion Urbana y Edificacion</t>
+          <t>Reglamento de Licencias de Habilitación Urbana y Edificación</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Ley de Regularizacion de Edificaciones</t>
+          <t>Ley de Regularización de Edificaciones</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Zonificacion de los Pantanos de Villa</t>
+          <t>Zonificación de los Pantanos de Villa</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Modulo de Compatibilidad SERNANP</t>
+          <t>Módulo de Compatibilidad SERNANP</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Ley General del Patrimonio Cultural de la Nacion</t>
+          <t>Ley General del Patrimonio Cultural de la Nación</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Reglamento del Registro Nacional de Obras de Construccion Civil (RENOCC)</t>
+          <t>Reglamento del Registro Nacional de Obras de Construcción Civil (RENOCC)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Beneficio de regularizacion de edificaciones en Surco (vencio 17-07-2025)</t>
+          <t>Beneficio de regularización de edificaciones en Surco (venció 17-07-2025)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Decreto Legislativo 1426 (modifica Ley 29090, art. 30 regularizacion)</t>
+          <t>Decreto Legislativo 1426 (modifica Ley 29090, art. 30 regularización)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Reglamento de Licencias de Habilitacion Urbana y Edificacion (D.S. 029-2019-VIVIENDA)</t>
+          <t>Reglamento de Licencias de Habilitación Urbana y Edificación (D.S. 029-2019-VIVIENDA)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>D.S. 146-2023-PCM: procedimientos estandarizados de licencias de habilitacion urbana y edificacion</t>
+          <t>D.S. 146-2023-PCM: procedimientos estandarizados de licencias de habilitación urbana y edificación</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3553,7 +3553,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Ley 30830 amplia la Ley 27157 hasta el 31-12-2016 (Rubio Leguia Normand)</t>
+          <t>Ley 30830 amplia la Ley 27157 hasta el 31-12-2016 (Rubio Leguía Normand)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>SUNARP: Declaratoria de fabrica y sus modalidades</t>
+          <t>SUNARP: Declaratoria de fábrica y sus modalidades</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Servicio de Publicidad Registral en Linea (Gana Mas)</t>
+          <t>Servicio de Publicidad Registral en Línea (Gana Más)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Infobae: proceso de formalizacion COFOPRI</t>
+          <t>Infobae: proceso de formalización COFOPRI</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>gob.pe: licencia de edificacion modalidad A</t>
+          <t>gob.pe: licencia de edificación modalidad A</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Tramites Peru: certificado de parametros urbanisticos</t>
+          <t>Trámites Perú: certificado de parámetros urbanísticos</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Municipalidad de Pueblo Libre: licencia de edificacion (plazos B, factibilidad)</t>
+          <t>Municipalidad de Pueblo Libre: licencia de edificación (plazos B, factibilidad)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Miraflores: licencia de edificacion (SGLEP)</t>
+          <t>Miraflores: licencia de edificación (SGLEP)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Lex Soluciones: regularizacion en Surco (Ord. 682-MSS) hasta 17-07-2025</t>
+          <t>Lex Soluciones: regularización en Surco (Ord. 682-MSS) hasta 17-07-2025</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Chorrillos: anexo zonificacion Pantanos de Villa (Ord. 184-MML)</t>
+          <t>Chorrillos: anexo zonificación Pantanos de Villa (Ord. 184-MML)</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Villa El Salvador: licencia de edificacion</t>
+          <t>Villa El Salvador: licencia de edificación</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>gob.pe: opinion ambiental PROHVILLA</t>
+          <t>gob.pe: opinión ambiental PROHVILLA</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>R.P. 049-2023-SERNANP: Modulo de Compatibilidad</t>
+          <t>R.P. 049-2023-SERNANP: Módulo de Compatibilidad</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>MTPE: registros de construccion civil</t>
+          <t>MTPE: registros de construcción civil</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Fondo MiVivienda: construccion en sitio propio</t>
+          <t>Fondo MiVivienda: construcción en sitio propio</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>FCR/ONP 2024: Banco de Materiales en liquidacion</t>
+          <t>FCR/ONP 2024: Banco de Materiales en liquidación</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Guia gob.pe: Plataforma de Interoperabilidad del Estado</t>
+          <t>Guía gob.pe: Plataforma de Interoperabilidad del Estado</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Datos Abiertos: resoluciones de licencias de edificacion MML</t>
+          <t>Datos Abiertos: resoluciones de licencias de edificación MML</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -4523,12 +4523,12 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Saneamiento fisico-legal y titularidad</t>
+          <t>Saneamiento físico-legal y titularidad</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Convertir la posesion o el contrato en propiedad inscrita en SUNARP.</t>
+          <t>Convertir la posesión o el contrato en propiedad inscrita en SUNARP.</t>
         </is>
       </c>
       <c r="E2" s="6" t="b">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Parametros urbanisticos, factibilidades y anteproyecto: definen que y cuanto se puede construir.</t>
+          <t>Parámetros urbanísticos, factibilidades y anteproyecto: definen qué y cuánto se puede construir.</t>
         </is>
       </c>
       <c r="E3" s="6" t="b">
@@ -4569,12 +4569,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Regularizacion de lo construido</t>
+          <t>Regularización de lo construido</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Solo si ya existe construccion sin licencia o sin declarar.</t>
+          <t>Solo si ya existe construcción sin licencia o sin declarar.</t>
         </is>
       </c>
       <c r="E4" s="6" t="b">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Solo si el predio esta en zona especial (Pantanos de Villa, ANP, zona monumental) o el proyecto lo exige.</t>
+          <t>Solo si el predio está en zona especial (Pantanos de Villa, ANP, zona monumental) o el proyecto lo exige.</t>
         </is>
       </c>
       <c r="E5" s="6" t="b">
@@ -4615,12 +4615,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion</t>
+          <t>Licencia de edificación</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Modalidad A, B, C o D segun tamano y uso.</t>
+          <t>Modalidad A, B, C o D según tamaño y uso.</t>
         </is>
       </c>
       <c r="E6" s="6" t="b">
@@ -4638,12 +4638,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Inicio y ejecucion de obra</t>
+          <t>Inicio y ejecución de obra</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Comunicacion de inicio, verificaciones tecnicas, seguros y obligaciones laborales.</t>
+          <t>Comunicación de inicio, verificaciones técnicas, seguros y obligaciones laborales.</t>
         </is>
       </c>
       <c r="E7" s="6" t="b">
@@ -4661,12 +4661,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra, declaratoria e inscripcion</t>
+          <t>Conformidad de obra, declaratoria e inscripción</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Cierre legal: conformidad municipal, inscripcion en SUNARP y actualizacion predial.</t>
+          <t>Cierre legal: conformidad municipal, inscripción en SUNARP y actualización predial.</t>
         </is>
       </c>
       <c r="E8" s="6" t="b">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Verifica titularidad, cargas y gravamenes antes de comprar o iniciar.</t>
+          <t>Verifica titularidad, cargas y gravámenes antes de comprar o iniciar.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -4840,7 +4840,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Segun SUNARP</t>
+          <t>Según SUNARP</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Copia de la partida; la licencia exige antiguedad maxima de 30 dias.</t>
+          <t>Copia de la partida; la licencia exige antigüedad máxima de 30 días.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -4925,7 +4925,7 @@
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Inmediata en linea</t>
+          <t>Inmediata en línea</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -4937,7 +4937,7 @@
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>Publicidad registral en linea: S/ 5 por asiento/pagina</t>
+          <t>Publicidad registral en línea: S/ 5 por asiento/página</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Escritura publica de compraventa</t>
+          <t>Escritura pública de compraventa</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>El notario eleva la minuta a escritura publica y la presenta a SUNARP por SID-Sunarp.</t>
+          <t>El notario eleva la minuta a escritura pública y la presenta a SUNARP por SID-Sunarp.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -5010,7 +5010,7 @@
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Segun notaria</t>
+          <t>Según notaría</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de compraventa</t>
+          <t>Inscripción de compraventa</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Calificacion registral e inscripcion de la transferencia.</t>
+          <t>Calificación registral e inscripción de la transferencia.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -5109,7 +5109,7 @@
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Derecho de calificacion; mas derecho de inscripcion segun valor (usar Calculadora Registral)</t>
+          <t>Derecho de calificación; más derecho de inscripción según valor (usar Calculadora Registral)</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Formalizacion de la propiedad (COFOPRI)</t>
+          <t>Formalización de la propiedad (COFOPRI)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Titulo gratuito para posesiones informales: terreno estatal ocupado hasta el 31-12-2021; privado con posesion pacifica de mas de 10 anos.</t>
+          <t>Título gratuito para posesiones informales: terreno estatal ocupado hasta el 31-12-2021; privado con posesión pacífica de más de 10 años.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -5267,7 +5267,7 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Proceso por campanas</t>
+          <t>Proceso por campañas</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Prescripcion adquisitiva de dominio</t>
+          <t>Prescripción adquisitiva de dominio</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Via notarial o judicial para quien posee como propietario por mas de 10 anos.</t>
+          <t>Vía notarial o judicial para quien posee como propietario por más de 10 años.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -5350,7 +5350,7 @@
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Meses; varia por caso</t>
+          <t>Meses; varía por caso</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Sucesion intestada</t>
+          <t>Sucesión intestada</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Declara herederos cuando el titular fallecio sin testamento; luego se inscribe en SUNARP.</t>
+          <t>Declara herederos cuando el titular falleció sin testamento; luego se inscribe en SUNARP.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Subdivision de lote</t>
+          <t>Subdivisión de lote</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Independizacion registral</t>
+          <t>Independización registral</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -5608,7 +5608,7 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>S/ 89-99 por unidad resultante + calificacion</t>
+          <t>S/ 89-99 por unidad resultante + calificación</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Parametros Urbanisticos y Edificatorios</t>
+          <t>Certificado de Parámetros Urbanísticos y Edificatorios</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Zonificacion, altura, retiros, area libre, densidad y estacionamientos del predio.</t>
+          <t>Zonificación, altura, retiros, área libre, densidad y estacionamientos del predio.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Zonificacion y Vias</t>
+          <t>Certificado de Zonificación y Vías</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Uso de suelo y seccion vial (principalmente habilitaciones urbanas).</t>
+          <t>Uso de suelo y sección vial (principalmente habilitaciones urbanas).</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Factibilidad de agua y desague</t>
+          <t>Factibilidad de agua y desagüe</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Factibilidad electrica</t>
+          <t>Factibilidad eléctrica</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -5993,7 +5993,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Asignacion / certificado de numeracion</t>
+          <t>Asignación / certificado de numeración</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Numeracion municipal del predio.</t>
+          <t>Numeración municipal del predio.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Revision del diseno antes del expediente completo; reduce observaciones.</t>
+          <t>Revisión del diseño antes del expediente completo; reduce observaciones.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Declaratoria de fabrica por regularizacion (Ley 27157)</t>
+          <t>Declaratoria de fábrica por regularización (Ley 27157)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -6183,7 +6183,7 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>S/ 41-50 fijo + 3/1000 del valor de la construccion</t>
+          <t>S/ 41-50 fijo + 3/1000 del valor de la construcción</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion en via de regularizacion</t>
+          <t>Licencia de edificación en vía de regularización</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Beneficio municipal de regularizacion (por ordenanza temporal)</t>
+          <t>Beneficio municipal de regularización (por ordenanza temporal)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Para obras posteriores al 17-09-2018 solo si el distrito tiene una ordenanza vigente. Ej.: Surco Ord. 682-MSS (obras 18-09-2018 a 31-12-2022), vencio el 17-07-2025.</t>
+          <t>Para obras posteriores al 17-09-2018 solo si el distrito tiene una ordenanza vigente. Ej.: Surco Ord. 682-MSS (obras 18-09-2018 a 31-12-2022), venció el 17-07-2025.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -6350,7 +6350,7 @@
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>Segun ordenanza</t>
+          <t>Según ordenanza</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Opinion ambiental PROHVILLA</t>
+          <t>Opinión ambiental PROHVILLA</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -6423,7 +6423,7 @@
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Suele demorar; en el caso real de referencia fue la etapa mas larga</t>
+          <t>Suele demorar; en el caso real de referencia fue la etapa más larga</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -6435,7 +6435,7 @@
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>Tasa segun TUPA MML/PROHVILLA</t>
+          <t>Tasa según TUPA MML/PROHVILLA</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Compatibilidad y opinion tecnica previa vinculante SERNANP</t>
+          <t>Compatibilidad y opinión técnica previa vinculante SERNANP</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Actividades en areas naturales protegidas de administracion nacional o su zona de amortiguamiento.</t>
+          <t>Actividades en áreas naturales protegidas de administración nacional o su zona de amortiguamiento.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -6516,7 +6516,7 @@
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Segun SERNANP</t>
+          <t>Según SERNANP</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Autorizacion del Ministerio de Cultura</t>
+          <t>Autorización del Ministerio de Cultura</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -6730,13 +6730,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Certificacion ambiental</t>
+          <t>Certificación ambiental</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Segun tipo y escala del proyecto (C/D).</t>
+          <t>Según tipo y escala del proyecto (C/D).</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad A (aprobacion automatica)</t>
+          <t>Licencia de edificación - Modalidad A (aprobación automática)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Vivienda unifamiliar nueva hasta 120 m2; ampliacion hasta 200 m2 totales; remodelacion sin cambio estructural; cercos de mas de 20 m; demolicion hasta 3 pisos; obras menores.</t>
+          <t>Vivienda unifamiliar nueva hasta 120 m²; ampliación hasta 200 m² totales; remodelación sin cambio estructural; cercos de más de 20 m; demolición hasta 3 pisos; obras menores.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Licencia al ingreso; verificacion administrativa en 10 dias habiles</t>
+          <t>Licencia al ingreso; verificación administrativa en 10 días hábiles</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad B (evaluacion municipal)</t>
+          <t>Licencia de edificación - Modalidad B (evaluación municipal)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -6904,7 +6904,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Vivienda hasta 5 pisos y hasta 3,000 m2; ampliaciones o remodelaciones con cambio estructural; demolicion parcial.</t>
+          <t>Vivienda hasta 5 pisos y hasta 3,000 m²; ampliaciones o remodelaciones con cambio estructural; demolición parcial.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>15 dias habiles (Pueblo Libre, La Molina)</t>
+          <t>15 días hábiles (Pueblo Libre, La Molina)</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad B (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad B (revisores urbanos)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Mismo alcance que B; el proyecto llega con informe tecnico favorable de revisores urbanos y la municipalidad cobra una tasa menor.</t>
+          <t>Mismo alcance que B; el proyecto llega con informe técnico favorable de revisores urbanos y la municipalidad cobra una tasa menor.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad C (comision tecnica)</t>
+          <t>Licencia de edificación - Modalidad C (comisión técnica)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Vivienda multifamiliar de mas de 5 pisos o mas de 3,000 m2; usos distintos a vivienda; uso mixto; patrimonio cultural; comercio hasta 30,000 m2; mercados hasta 15,000 m2.</t>
+          <t>Vivienda multifamiliar de más de 5 pisos o más de 3,000 m²; usos distintos a vivienda; uso mixto; patrimonio cultural; comercio hasta 30,000 m²; mercados hasta 15,000 m².</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Hasta 25 dias habiles de evaluacion de comision (La Molina, flujo anterior)</t>
+          <t>Hasta 25 días hábiles de evaluación de comisión (La Molina, flujo anterior)</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad C (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad C (revisores urbanos)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad D (comision tecnica)</t>
+          <t>Licencia de edificación - Modalidad D (comisión técnica)</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Industria; comercio de mas de 30,000 m2; mercados de mas de 15,000 m2; educacion, salud, hospedaje.</t>
+          <t>Industria; comercio de más de 30,000 m²; mercados de más de 15,000 m²; educación, salud, hospedaje.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad D (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad D (revisores urbanos)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Modificacion de proyecto (antes o despues de la licencia; sustancial o no sustancial)</t>
+          <t>Modificación de proyecto (antes o después de la licencia; sustancial o no sustancial)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Prorroga de licencia (12 meses)</t>
+          <t>Prórroga de licencia (12 meses)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Unica prorroga; debe pedirse antes del vencimiento de los 36 meses.</t>
+          <t>Única prórroga; debe pedirse antes del vencimiento de los 36 meses.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Revalidacion de licencia</t>
+          <t>Revalidación de licencia</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Cuando la licencia ya vencio.</t>
+          <t>Cuando la licencia ya venció.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Comunicacion de inicio de obra (Anexo H)</t>
+          <t>Comunicación de inicio de obra (Anexo H)</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Aviso formal antes de iniciar, con cronograma de verificaciones tecnicas.</t>
+          <t>Aviso formal antes de iniciar, con cronograma de verificaciones técnicas.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -7678,7 +7678,7 @@
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>Segun TUPA; en varios distritos sin costo</t>
+          <t>Según TUPA; en varios distritos sin costo</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Verificaciones tecnicas durante la obra</t>
+          <t>Verificaciones técnicas durante la obra</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Visitas en hitos (cimentacion, albanileria, techos). Desvios respecto a planos pueden derivar en paralizacion.</t>
+          <t>Visitas en hitos (cimentación, albañilería, techos). Desvíos respecto a planos pueden derivar en paralización.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -7763,7 +7763,7 @@
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="inlineStr">
         <is>
-          <t>Segun TUPA</t>
+          <t>Según TUPA</t>
         </is>
       </c>
       <c r="M37" s="6" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Contratar poliza CAR o de responsabilidad civil</t>
+          <t>Contratar póliza CAR o de responsabilidad civil</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -7825,7 +7825,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Cobertura por danos a terceros durante toda la obra (C y D, y segun reglamento).</t>
+          <t>Cobertura por daños a terceros durante toda la obra (C y D, y según reglamento).</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de la obra en RENOCC</t>
+          <t>Inscripción de la obra en RENOCC</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Obligatoria para obras de construccion civil de mas de 50 UIT (S/ 275,000 en 2026).</t>
+          <t>Obligatoria para obras de construcción civil de más de 50 UIT (S/ 275,000 en 2026).</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -7925,7 +7925,7 @@
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>Segun MTPE</t>
+          <t>Según MTPE</t>
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Registro de trabajadores de construccion civil (RETCC)</t>
+          <t>Registro de trabajadores de construcción civil (RETCC)</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Trabajadores del regimen de construccion civil deben estar registrados.</t>
+          <t>Trabajadores del régimen de construcción civil deben estar registrados.</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -8006,7 +8006,7 @@
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>Segun MTPE</t>
+          <t>Según MTPE</t>
         </is>
       </c>
       <c r="M40" s="6" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Obligatorio para actividades de riesgo, incluida construccion.</t>
+          <t>Obligatorio para actividades de riesgo, incluida construcción.</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Aporte de los obreros de construccion civil, retenido por el empleador.</t>
+          <t>Aporte de los obreros de construcción civil, retenido por el empleador.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -8172,7 +8172,7 @@
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>Porcentaje del jornal basico por confirmar</t>
+          <t>Porcentaje del jornal básico por confirmar</t>
         </is>
       </c>
       <c r="M42" s="6" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Contribucion sobre ingresos por obras de construccion. Confirmar si aplica a autoconstruccion familiar.</t>
+          <t>Contribución sobre ingresos por obras de construcción. Confirmar si aplica a autoconstrucción familiar.</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Cartel de obra con numero de licencia</t>
+          <t>Cartel de obra con número de licencia</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Visible durante toda la ejecucion.</t>
+          <t>Visible durante toda la ejecución.</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -8386,7 +8386,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra y declaratoria de edificacion sin variaciones</t>
+          <t>Conformidad de obra y declaratoria de edificación sin variaciones</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra y declaratoria de edificacion con variaciones</t>
+          <t>Conformidad de obra y declaratoria de edificación con variaciones</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Predeclaratoria de edificacion</t>
+          <t>Predeclaratoria de edificación</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de la declaratoria de edificacion</t>
+          <t>Inscripción de la declaratoria de edificación</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -8738,7 +8738,7 @@
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Calificacion (~S/ 41-50) + 3/1000 del valor de la obra</t>
+          <t>Calificación (~S/ 41-50) + 3/1000 del valor de la obra</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de reglamento interno e independizacion de unidades</t>
+          <t>Inscripción de reglamento interno e independización de unidades</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Multifamiliares: cada departamento, estacionamiento o deposito con partida propia.</t>
+          <t>Multifamiliares: cada departamento, estacionamiento o depósito con partida propia.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -8823,7 +8823,7 @@
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>S/ 89-99 por unidad + calificacion</t>
+          <t>S/ 89-99 por unidad + calificación</t>
         </is>
       </c>
       <c r="L50" s="6" t="n"/>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Actualizar declaracion jurada del impuesto predial</t>
+          <t>Actualizar declaración jurada del impuesto predial</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -9012,7 +9012,7 @@
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Identificacion.</t>
+          <t>Identificación.</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
@@ -9040,7 +9040,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Punto de partida cuando la propiedad no esta inscrita.</t>
+          <t>Punto de partida cuando la propiedad no está inscrita.</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -9057,7 +9057,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Escritura publica</t>
+          <t>Escritura pública</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -9096,7 +9096,7 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Muestra cargas, gravamenes y titularidad.</t>
+          <t>Muestra cargas, gravámenes y titularidad.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>La licencia exige una copia con antiguedad maxima de 30 dias.</t>
+          <t>La licencia exige una copia con antigüedad máxima de 30 días.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Titulo de propiedad COFOPRI inscrito</t>
+          <t>Título de propiedad COFOPRI inscrito</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -9154,7 +9154,7 @@
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Resultado de la formalizacion.</t>
+          <t>Resultado de la formalización.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Sucesion intestada o testamento inscrito</t>
+          <t>Sucesión intestada o testamento inscrito</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -9182,7 +9182,7 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Necesario si el titular registral fallecio.</t>
+          <t>Necesario si el titular registral falleció.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Si tramita un representante o persona juridica.</t>
+          <t>Si tramita un representante o persona jurídica.</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -9229,7 +9229,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Parametros Urbanisticos y Edificatorios</t>
+          <t>Certificado de Parámetros Urbanísticos y Edificatorios</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Zonificacion y Vias</t>
+          <t>Certificado de Zonificación y Vías</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Certificado de factibilidad de agua y desague</t>
+          <t>Certificado de factibilidad de agua y desagüe</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Vigencia 36 meses segun Pueblo Libre.</t>
+          <t>Vigencia 36 meses según Pueblo Libre.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Certificado de factibilidad electrica</t>
+          <t>Certificado de factibilidad eléctrica</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Luz del Sur o Enel segun zona. Vigencia por confirmar.</t>
+          <t>Luz del Sur o Enel según zona. Vigencia por confirmar.</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Formulario Unico de Edificaciones (FUE)</t>
+          <t>Formulario Único de Edificaciones (FUE)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Anexos del FUE (A: condominos, B, D: autoliquidacion, H: inicio de obra)</t>
+          <t>Anexos del FUE (A: condóminos, B, D: autoliquidación, H: inicio de obra)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -9384,7 +9384,7 @@
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Anexo H = comunicacion de inicio de obra.</t>
+          <t>Anexo H = comunicación de inicio de obra.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Plano de ubicacion y localizacion</t>
+          <t>Plano de ubicación y localización</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -9497,7 +9497,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Planos de instalaciones electricas</t>
+          <t>Planos de instalaciones eléctricas</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -9521,14 +9521,14 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Estudio de Mecanica de Suelos (EMS)</t>
+          <t>Estudio de Mecánica de Suelos (EMS)</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Surco: obligatorio desde 4 pisos o mas de 500 m2 en primer piso.</t>
+          <t>Surco: obligatorio desde 4 pisos o más de 500 m² en primer piso.</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -9552,7 +9552,7 @@
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Excavaciones de mas de 2 m.</t>
+          <t>Excavaciones de más de 2 m.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -9569,14 +9569,14 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Planos de seguridad y evacuacion</t>
+          <t>Planos de seguridad y evacuación</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Edificios de mas de 5 pisos y usos con afluencia de publico.</t>
+          <t>Edificios de más de 5 pisos y usos con afluencia de público.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Poliza CAR o de responsabilidad civil</t>
+          <t>Póliza CAR o de responsabilidad civil</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -9697,14 +9697,14 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Certificacion ambiental</t>
+          <t>Certificación ambiental</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Segun tipo de proyecto (C/D).</t>
+          <t>Según tipo de proyecto (C/D).</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -9721,7 +9721,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Opinion ambiental de PROHVILLA</t>
+          <t>Opinión ambiental de PROHVILLA</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Compatibilidad / opinion tecnica previa vinculante SERNANP</t>
+          <t>Compatibilidad / opinión técnica previa vinculante SERNANP</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Autorizacion del Ministerio de Cultura</t>
+          <t>Autorización del Ministerio de Cultura</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Resolucion de licencia de edificacion</t>
+          <t>Resolución de licencia de edificación</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -9876,7 +9876,7 @@
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Declaratoria de fabrica por regularizacion.</t>
+          <t>Declaratoria de fábrica por regularización.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Informe tecnico del verificador responsable</t>
+          <t>Informe técnico del verificador responsable</t>
         </is>
       </c>
       <c r="C35" s="6" t="n"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Cronograma de visitas de verificacion tecnica</t>
+          <t>Cronograma de visitas de verificación técnica</t>
         </is>
       </c>
       <c r="C37" s="6" t="n"/>
@@ -9969,7 +9969,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Poliza SCTR (salud y pension)</t>
+          <t>Póliza SCTR (salud y pensión)</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -9980,7 +9980,7 @@
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Obligatoria para trabajadores de construccion civil.</t>
+          <t>Obligatoria para trabajadores de construcción civil.</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Constancia de inscripcion de obra en RENOCC</t>
+          <t>Constancia de inscripción de obra en RENOCC</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -10008,7 +10008,7 @@
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Obras de mas de 50 UIT.</t>
+          <t>Obras de más de 50 UIT.</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Resolucion de conformidad de obra y declaratoria de edificacion</t>
+          <t>Resolución de conformidad de obra y declaratoria de edificación</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Autoriza la inscripcion registral.</t>
+          <t>Autoriza la inscripción registral.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -10084,7 +10084,7 @@
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Multifamiliares / propiedad exclusiva y comun.</t>
+          <t>Multifamiliares / propiedad exclusiva y común.</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -10101,7 +10101,7 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Declaracion jurada de autoavaluo actualizada</t>
+          <t>Declaración jurada de autoavalúo actualizada</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Superintendencia Nacional de los Registros Publicos</t>
+          <t>Superintendencia Nacional de los Registros Públicos</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>SID-Sunarp (notarios), Publicidad Registral en Linea, Siguelo, Alerta Registral</t>
+          <t>SID-Sunarp (notarios), Publicidad Registral en Línea, Síguelo, Alerta Registral</t>
         </is>
       </c>
     </row>
@@ -10227,7 +10227,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Notaria publica</t>
+          <t>Notaría pública</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -10248,7 +10248,7 @@
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Presencial; presenta a SUNARP via SID-Sunarp</t>
+          <t>Presencial; presenta a SUNARP vía SID-Sunarp</t>
         </is>
       </c>
     </row>
@@ -10260,7 +10260,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Organismo de Formalizacion de la Propiedad Informal</t>
+          <t>Organismo de Formalización de la Propiedad Informal</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -10285,7 +10285,7 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Campanas y oficinas</t>
+          <t>Campañas y oficinas</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Mesa de partes electronica</t>
+          <t>Mesa de partes electrónica</t>
         </is>
       </c>
     </row>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Municipalidad distrital (segun ubicacion del predio)</t>
+          <t>Municipalidad distrital (según ubicación del predio)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -10355,7 +10355,7 @@
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Varia por distrito: ver distritos.json</t>
+          <t>Varía por distrito: ver distritos.json</t>
         </is>
       </c>
     </row>
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Servicio de Administracion Tributaria de Lima</t>
+          <t>Servicio de Administración Tributaria de Lima</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tramite en gob.pe</t>
+          <t>Trámite en gob.pe</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Servicio Nacional de Areas Naturales Protegidas</t>
+          <t>Servicio Nacional de Áreas Naturales Protegidas</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -10503,7 +10503,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Modulo de Compatibilidad en linea</t>
+          <t>Módulo de Compatibilidad en línea</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de Vivienda, Construccion y Saneamiento</t>
+          <t>Ministerio de Vivienda, Construcción y Saneamiento</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Plataforma de tramites digitales</t>
+          <t>Plataforma de trámites digitales</t>
         </is>
       </c>
     </row>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Postulacion en linea, 0800-12-200</t>
+          <t>Postulación en línea, 0800-12-200</t>
         </is>
       </c>
     </row>
@@ -10626,7 +10626,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de Trabajo y Promocion del Empleo</t>
+          <t>Ministerio de Trabajo y Promoción del Empleo</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Registros de construccion civil en linea</t>
+          <t>Registros de construcción civil en línea</t>
         </is>
       </c>
     </row>
@@ -10725,7 +10725,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Atencion virtual; atiende Lima Sur y Este</t>
+          <t>Atención virtual; atiende Lima Sur y Este</t>
         </is>
       </c>
     </row>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Enel Distribucion Peru</t>
+          <t>Enel Distribución Perú</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Atencion virtual; atiende Lima Norte y Oeste</t>
+          <t>Atención virtual; atiende Lima Norte y Oeste</t>
         </is>
       </c>
     </row>
@@ -10774,7 +10774,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Colegio de Arquitectos / Colegio de Ingenieros del Peru</t>
+          <t>Colegio de Arquitectos / Colegio de Ingenieros del Perú</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -10795,7 +10795,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Delegados en comisiones tecnicas; habilidad profesional</t>
+          <t>Delegados en comisiones técnicas; habilidad profesional</t>
         </is>
       </c>
     </row>
@@ -10828,7 +10828,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Alternativa a la municipalidad/comision en B, C y D</t>
+          <t>Alternativa a la municipalidad/comisión en B, C y D</t>
         </is>
       </c>
     </row>
@@ -10840,7 +10840,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Compania de seguros</t>
+          <t>Compañía de seguros</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -10861,7 +10861,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Poliza CAR / responsabilidad civil / SCTR</t>
+          <t>Póliza CAR / responsabilidad civil / SCTR</t>
         </is>
       </c>
     </row>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Servicio Nacional de Capacitacion para la Industria de la Construccion</t>
+          <t>Servicio Nacional de Capacitación para la Industria de la Construcción</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Declaracion y pago</t>
+          <t>Declaración y pago</t>
         </is>
       </c>
     </row>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Fondo de Vivienda del Trabajador de Construccion Civil</t>
+          <t>Fondo de Vivienda del Trabajador de Construcción Civil</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Retencion por el empleador</t>
+          <t>Retención por el empleador</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Participan en comision tecnica</t>
+          <t>Participan en comisión técnica</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>El PDF publicado no expone montos legibles de edificacion; confirmar TUPA vigente y su adecuacion al D.S. 146-2023-PCM.</t>
+          <t>El PDF publicado no expone montos legibles de edificación; confirmar TUPA vigente y su adecuación al D.S. 146-2023-PCM.</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -11158,7 +11158,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>TUPA publicado el 27-09-2024 (220 procedimientos). Montos de licencias tomados de la version 2022: confirmar.</t>
+          <t>TUPA publicado el 27-09-2024 (220 procedimientos). Montos de licencias tomados de la versión 2022: confirmar.</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>TUPA 2025 ratificado por la MML; 123 procedimientos de HU y edificacion adecuados al D.S. 146-2023-PCM (vigente desde 22-06-2024). Montos por extraer del anexo.</t>
+          <t>TUPA 2025 ratificado por la MML; 123 procedimientos de HU y edificación adecuados al D.S. 146-2023-PCM (vigente desde 22-06-2024). Montos por extraer del anexo.</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Distrito de referencia: unico con tasas completas extraidas (TUPA 2025, UIT 5,350).</t>
+          <t>Distrito de referencia: único con tasas completas extraídas (TUPA 2025, UIT 5,350).</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>Monto atipicamente bajo en la extraccion: confirmar</t>
+          <t>Monto atípicamente bajo en la extracción: confirmar</t>
         </is>
       </c>
     </row>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>Rango 2022: S/ 56.10 a 122.20 segun submodalidad</t>
+          <t>Rango 2022: S/ 56.10 a 122.20 según submodalidad</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13480,7 @@
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13524,7 +13524,7 @@
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13568,7 +13568,7 @@
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13612,7 +13612,7 @@
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13656,7 +13656,7 @@
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13700,7 +13700,7 @@
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13744,7 +13744,7 @@
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13832,7 +13832,7 @@
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13876,7 +13876,7 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13920,7 +13920,7 @@
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13964,7 +13964,7 @@
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14008,7 +14008,7 @@
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14052,7 +14052,7 @@
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14140,7 +14140,7 @@
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14184,7 +14184,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14228,7 +14228,7 @@
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14595,7 +14595,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>{"alturas_pisos": "2 a 4 (zonas residenciales RDMB, RDB, RDM)", "area_libre_pct": "30 a 60", "retiro_frontal_m": "5 a 25", "otros": "Arborizacion obligatoria; restriccion de subdivisiones; ZHR max. 2 pisos; IE max. 1 piso"}</t>
+          <t>{"alturas_pisos": "2 a 4 (zonas residenciales RDMB, RDB, RDM)", "area_libre_pct": "30 a 60", "retiro_frontal_m": "5 a 25", "otros": "Arborización obligatoria; restricción de subdivisiones; ZHR max. 2 pisos; IE max. 1 piso"}</t>
         </is>
       </c>
       <c r="I2" s="6" t="n"/>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Area Natural Protegida nacional o su zona de amortiguamiento</t>
+          <t>Área Natural Protegida nacional o su zona de amortiguamiento</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -14803,7 +14803,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Techo Propio - Construccion en Sitio Propio</t>
+          <t>Techo Propio - Construcción en Sitio Propio</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>["Ingreso familiar mensual hasta S/ 2,706", "Ahorro minimo S/ 2,475", "Terreno o aires inscritos en SUNARP", "No tener otra propiedad ni beneficio previo", "Grupo familiar constituido"]</t>
+          <t>["Ingreso familiar mensual hasta S/ 2,706", "Ahorro mínimo S/ 2,475", "Terreno o aires inscritos en SUNARP", "No tener otra propiedad ni beneficio previo", "Grupo familiar constituido"]</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -14851,7 +14851,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Techo Propio - Adquisicion de Vivienda Nueva</t>
+          <t>Techo Propio - Adquisición de Vivienda Nueva</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Segun convocatoria</t>
+          <t>Según convocatoria</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Creditos MiVivienda y productos de construccion</t>
+          <t>Créditos MiVivienda y productos de construcción</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Credito hipotecario via bancos y cajas</t>
+          <t>Crédito hipotecario vía bancos y cajas</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Formalizacion gratuita COFOPRI</t>
+          <t>Formalización gratuita COFOPRI</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -14960,12 +14960,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Titulo de propiedad gratuito inscrito</t>
+          <t>Título de propiedad gratuito inscrito</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>["Terreno estatal ocupado hasta 31-12-2021 o privado con posesion de mas de 10 anos"]</t>
+          <t>["Terreno estatal ocupado hasta 31-12-2021 o privado con posesión de más de 10 años"]</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>En liquidacion: no otorga creditos nuevos</t>
+          <t>En liquidación: no otorga créditos nuevos</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
data: corrige tildes y signos de apertura en los textos visibles (#4)
Solo cambian textos mostrados al usuario; ids, valores de opciones, condiciones, URLs, siglas y codigos quedan iguales. El motor da el mismo resultado (6/6); en resultados-motor.json solo cambian los mensajes de alerta.
</commit_message>
<xml_diff>
--- a/data/ruta-obra.xlsx
+++ b/data/ruta-obra.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Informacion referencial. No es asesoria legal. Montos y plazos deben confirmarse en el TUPA vigente de cada entidad antes de presentar un tramite.</t>
+          <t>Información referencial. No es asesoría legal. Montos y plazos deben confirmarse en el TUPA vigente de cada entidad antes de presentar un trámite.</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dato leido en la fuente oficial citada.</t>
+          <t>Dato leído en la fuente oficial citada.</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dato oficial de una version anterior del TUPA o norma; confirmar vigencia.</t>
+          <t>Dato oficial de una versión anterior del TUPA o norma; confirmar vigencia.</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Como esta la propiedad del terreno hoy?</t>
+          <t>¿Cómo está la propiedad del terreno hoy?</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "inscrito", "etiqueta": "Inscrita en SUNARP a mi nombre"}, {"valor": "compraventa_no_inscrita", "etiqueta": "Tengo contrato o minuta de compraventa, sin inscribir"}, {"valor": "posesion_estatal", "etiqueta": "Posesion en terreno del Estado, sin titulo"}, {"valor": "posesion_privada", "etiqueta": "Posesion en terreno privado por mas de 10 anos, sin titulo"}, {"valor": "herencia", "etiqueta": "Heredada, a nombre de un familiar fallecido"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "inscrito", "etiqueta": "Inscrita en SUNARP a mi nombre"}, {"valor": "compraventa_no_inscrita", "etiqueta": "Tengo contrato o minuta de compraventa, sin inscribir"}, {"valor": "posesion_estatal", "etiqueta": "Posesión en terreno del Estado, sin título"}, {"valor": "posesion_privada", "etiqueta": "Posesión en terreno privado por más de 10 años, sin título"}, {"valor": "herencia", "etiqueta": "Heredada, a nombre de un familiar fallecido"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
@@ -687,7 +687,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>El predio tiene partida registral propia (no es parte de un lote mayor)?</t>
+          <t>¿El predio tiene partida registral propia (no es parte de un lote mayor)?</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No, es parte de un lote mayor"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No, es parte de un lote mayor"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
@@ -715,7 +715,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Ya hay algo construido en el terreno?</t>
+          <t>¿Ya hay algo construido en el terreno?</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "no", "etiqueta": "No, terreno libre"}, {"valor": "si_declarada", "etiqueta": "Si, y esta declarada en SUNARP"}, {"valor": "si_sin_declarar", "etiqueta": "Si, pero sin licencia o sin declarar"}]</t>
+          <t>[{"valor": "no", "etiqueta": "No, terreno libre"}, {"valor": "si_declarada", "etiqueta": "Sí, y está declarada en SUNARP"}, {"valor": "si_sin_declarar", "etiqueta": "Sí, pero sin licencia o sin declarar"}]</t>
         </is>
       </c>
       <c r="F4" s="6" t="n"/>
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Cuando se termino lo construido sin licencia?</t>
+          <t>¿Cuándo se terminó lo construido sin licencia?</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "hasta_2016", "etiqueta": "Hasta el 31-12-2016"}, {"valor": "2017_sep2018", "etiqueta": "Entre el 01-01-2017 y el 17-09-2018"}, {"valor": "post_sep2018", "etiqueta": "Despues del 17-09-2018"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "hasta_2016", "etiqueta": "Hasta el 31-12-2016"}, {"valor": "2017_sep2018", "etiqueta": "Entre el 01-01-2017 y el 17-09-2018"}, {"valor": "post_sep2018", "etiqueta": "Después del 17-09-2018"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>En que distrito esta el predio?</t>
+          <t>¿En qué distrito está el predio?</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>El predio esta en alguna de estas zonas?</t>
+          <t>¿El predio está en alguna de estas zonas?</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "pantanos_villa", "etiqueta": "Cerca de los Pantanos de Villa"}, {"valor": "anp", "etiqueta": "Area natural protegida o su zona de amortiguamiento"}, {"valor": "monumental", "etiqueta": "Zona monumental o inmueble historico"}, {"valor": "ninguna", "etiqueta": "Ninguna"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "pantanos_villa", "etiqueta": "Cerca de los Pantanos de Villa"}, {"valor": "anp", "etiqueta": "Área natural protegida o su zona de amortiguamiento"}, {"valor": "monumental", "etiqueta": "Zona monumental o inmueble histórico"}, {"valor": "ninguna", "etiqueta": "Ninguna"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F7" s="6" t="n"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Que quieres hacer?</t>
+          <t>¿Qué quieres hacer?</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "obra_nueva", "etiqueta": "Construir desde cero"}, {"valor": "ampliacion", "etiqueta": "Ampliar (mas pisos o mas area)"}, {"valor": "remodelacion", "etiqueta": "Remodelar"}, {"valor": "demolicion", "etiqueta": "Demoler"}, {"valor": "cerco", "etiqueta": "Solo cerco perimetrico"}]</t>
+          <t>[{"valor": "obra_nueva", "etiqueta": "Construir desde cero"}, {"valor": "ampliacion", "etiqueta": "Ampliar (más pisos o más área)"}, {"valor": "remodelacion", "etiqueta": "Remodelar"}, {"valor": "demolicion", "etiqueta": "Demoler"}, {"valor": "cerco", "etiqueta": "Solo cerco perimétrico"}]</t>
         </is>
       </c>
       <c r="F8" s="6" t="n"/>
@@ -859,7 +859,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Para que uso?</t>
+          <t>¿Para qué uso?</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "vivienda_unifamiliar", "etiqueta": "Vivienda de una familia"}, {"valor": "vivienda_multifamiliar", "etiqueta": "Vivienda de varias familias / departamentos"}, {"valor": "comercio", "etiqueta": "Comercio u oficinas"}, {"valor": "mixto", "etiqueta": "Vivienda + comercio"}, {"valor": "industria", "etiqueta": "Industria"}, {"valor": "educacion_salud_hospedaje", "etiqueta": "Educacion, salud u hospedaje"}]</t>
+          <t>[{"valor": "vivienda_unifamiliar", "etiqueta": "Vivienda de una familia"}, {"valor": "vivienda_multifamiliar", "etiqueta": "Vivienda de varias familias / departamentos"}, {"valor": "comercio", "etiqueta": "Comercio u oficinas"}, {"valor": "mixto", "etiqueta": "Vivienda + comercio"}, {"valor": "industria", "etiqueta": "Industria"}, {"valor": "educacion_salud_hospedaje", "etiqueta": "Educación, salud u hospedaje"}]</t>
         </is>
       </c>
       <c r="F9" s="6" t="n"/>
@@ -887,7 +887,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Cuantos pisos tendra en total?</t>
+          <t>¿Cuántos pisos tendrá en total?</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Area techada total al terminar (m2)</t>
+          <t>Área techada total al terminar (m²)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>La obra modifica la estructura (columnas, vigas, losas)?</t>
+          <t>¿La obra modifica la estructura (columnas, vigas, losas)?</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}, {"valor": "no_se", "etiqueta": "No lo se"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}, {"valor": "no_se", "etiqueta": "No lo sé"}]</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Habra sotano o excavacion de mas de 2 m?</t>
+          <t>¿Habrá sótano o excavación de más de 2 m?</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}]</t>
         </is>
       </c>
       <c r="F13" s="6" t="n"/>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Como piensas financiarla?</t>
+          <t>¿Cómo piensas financiarla?</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "techo_propio", "etiqueta": "Bono Techo Propio"}, {"valor": "credito", "etiqueta": "Credito hipotecario / MiVivienda"}, {"valor": "propio", "etiqueta": "Recursos propios"}]</t>
+          <t>[{"valor": "techo_propio", "etiqueta": "Bono Techo Propio"}, {"valor": "credito", "etiqueta": "Crédito hipotecario / MiVivienda"}, {"valor": "propio", "etiqueta": "Recursos propios"}]</t>
         </is>
       </c>
       <c r="F15" s="6" t="n"/>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Contrataras maestro de obra y obreros?</t>
+          <t>¿Contratarás maestro de obra y obreros?</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>[{"valor": "si", "etiqueta": "Si"}, {"valor": "no", "etiqueta": "No"}]</t>
+          <t>[{"valor": "si", "etiqueta": "Sí"}, {"valor": "no", "etiqueta": "No"}]</t>
         </is>
       </c>
       <c r="F16" s="6" t="n"/>
@@ -2067,7 +2067,7 @@
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>Segun envergadura; confirmar con la municipalidad</t>
+          <t>Según envergadura; confirmar con la municipalidad</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>Lo construido despues del 17-09-2018 solo se regulariza si tu distrito tiene una ordenanza de beneficio vigente. Sin ella hay riesgo de multa o demolicion.</t>
+          <t>Lo construido después del 17-09-2018 solo se regulariza si tu distrito tiene una ordenanza de beneficio vigente. Sin ella hay riesgo de multa o demolición.</t>
         </is>
       </c>
       <c r="M40" s="6" t="n"/>
@@ -2515,7 +2515,7 @@
       </c>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>Necesitas opinion de PROHVILLA antes de la licencia. Suele ser la etapa mas larga: iniciala en paralelo con los documentos previos. Alturas de 2 a 4 pisos y area libre de 30% a 60% segun zona.</t>
+          <t>Necesitas opinión de PROHVILLA antes de la licencia. Suele ser la etapa más larga: iníciala en paralelo con los documentos previos. Alturas de 2 a 4 pisos y área libre de 30% a 60% según zona.</t>
         </is>
       </c>
       <c r="M41" s="6" t="n"/>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>Pide primero el certificado de parametros: indica si el predio esta en zona especial.</t>
+          <t>Pide primero el certificado de parámetros: indica si el predio está en zona especial.</t>
         </is>
       </c>
       <c r="M42" s="6" t="n"/>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="L43" s="6" t="inlineStr">
         <is>
-          <t>Excavaciones de mas de 2 m requieren plano de sostenimiento.</t>
+          <t>Excavaciones de más de 2 m requieren plano de sostenimiento.</t>
         </is>
       </c>
       <c r="M43" s="6" t="n"/>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="L45" s="6" t="inlineStr">
         <is>
-          <t>Tu distrito aun no tiene tasas cargadas: la ruta es valida (norma nacional), pero montos y canal deben confirmarse en su TUPA.</t>
+          <t>Tu distrito aún no tiene tasas cargadas: la ruta es válida (norma nacional), pero montos y canal deben confirmarse en su TUPA.</t>
         </is>
       </c>
       <c r="M45" s="6" t="n"/>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>La copia literal vence: la licencia exige maximo 30 dias de antiguedad.</t>
+          <t>La copia literal vence: la licencia exige máximo 30 días de antigüedad.</t>
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>El certificado de parametros vence (36 meses).</t>
+          <t>El certificado de parámetros vence (36 meses).</t>
         </is>
       </c>
       <c r="F3" s="6" t="n"/>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>La licencia vence (36 meses). Pide la prorroga de 12 meses ANTES del vencimiento.</t>
+          <t>La licencia vence (36 meses). Pide la prórroga de 12 meses ANTES del vencimiento.</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Tienes 5 dias habiles para subsanar observaciones (prorrogables 5 mas en algunos distritos).</t>
+          <t>Tienes 5 días hábiles para subsanar observaciones (prorrogables 5 más en algunos distritos).</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Ley de Regulacion de Habilitaciones Urbanas y de Edificaciones</t>
+          <t>Ley de Regulación de Habilitaciones Urbanas y de Edificaciones</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Modifica la Ley 29090 (regularizacion art. 30)</t>
+          <t>Modifica la Ley 29090 (regularización art. 30)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Reglamento de Licencias de Habilitacion Urbana y Edificacion</t>
+          <t>Reglamento de Licencias de Habilitación Urbana y Edificación</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Ley de Regularizacion de Edificaciones</t>
+          <t>Ley de Regularización de Edificaciones</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Zonificacion de los Pantanos de Villa</t>
+          <t>Zonificación de los Pantanos de Villa</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Modulo de Compatibilidad SERNANP</t>
+          <t>Módulo de Compatibilidad SERNANP</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Ley General del Patrimonio Cultural de la Nacion</t>
+          <t>Ley General del Patrimonio Cultural de la Nación</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Reglamento del Registro Nacional de Obras de Construccion Civil (RENOCC)</t>
+          <t>Reglamento del Registro Nacional de Obras de Construcción Civil (RENOCC)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Beneficio de regularizacion de edificaciones en Surco (vencio 17-07-2025)</t>
+          <t>Beneficio de regularización de edificaciones en Surco (venció 17-07-2025)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>regularizacion</t>
+          <t>regularización</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Decreto Legislativo 1426 (modifica Ley 29090, art. 30 regularizacion)</t>
+          <t>Decreto Legislativo 1426 (modifica Ley 29090, art. 30 regularización)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Reglamento de Licencias de Habilitacion Urbana y Edificacion (D.S. 029-2019-VIVIENDA)</t>
+          <t>Reglamento de Licencias de Habilitación Urbana y Edificación (D.S. 029-2019-VIVIENDA)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>D.S. 146-2023-PCM: procedimientos estandarizados de licencias de habilitacion urbana y edificacion</t>
+          <t>D.S. 146-2023-PCM: procedimientos estandarizados de licencias de habilitación urbana y edificación</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3553,7 +3553,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Ley 30830 amplia la Ley 27157 hasta el 31-12-2016 (Rubio Leguia Normand)</t>
+          <t>Ley 30830 amplia la Ley 27157 hasta el 31-12-2016 (Rubio Leguía Normand)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>SUNARP: Declaratoria de fabrica y sus modalidades</t>
+          <t>SUNARP: Declaratoria de fábrica y sus modalidades</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Servicio de Publicidad Registral en Linea (Gana Mas)</t>
+          <t>Servicio de Publicidad Registral en Línea (Gana Más)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Infobae: proceso de formalizacion COFOPRI</t>
+          <t>Infobae: proceso de formalización COFOPRI</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>gob.pe: licencia de edificacion modalidad A</t>
+          <t>gob.pe: licencia de edificación modalidad A</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Tramites Peru: certificado de parametros urbanisticos</t>
+          <t>Trámites Perú: certificado de parámetros urbanísticos</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Municipalidad de Pueblo Libre: licencia de edificacion (plazos B, factibilidad)</t>
+          <t>Municipalidad de Pueblo Libre: licencia de edificación (plazos B, factibilidad)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Miraflores: licencia de edificacion (SGLEP)</t>
+          <t>Miraflores: licencia de edificación (SGLEP)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Lex Soluciones: regularizacion en Surco (Ord. 682-MSS) hasta 17-07-2025</t>
+          <t>Lex Soluciones: regularización en Surco (Ord. 682-MSS) hasta 17-07-2025</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Chorrillos: anexo zonificacion Pantanos de Villa (Ord. 184-MML)</t>
+          <t>Chorrillos: anexo zonificación Pantanos de Villa (Ord. 184-MML)</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Villa El Salvador: licencia de edificacion</t>
+          <t>Villa El Salvador: licencia de edificación</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>gob.pe: opinion ambiental PROHVILLA</t>
+          <t>gob.pe: opinión ambiental PROHVILLA</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>R.P. 049-2023-SERNANP: Modulo de Compatibilidad</t>
+          <t>R.P. 049-2023-SERNANP: Módulo de Compatibilidad</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>MTPE: registros de construccion civil</t>
+          <t>MTPE: registros de construcción civil</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Fondo MiVivienda: construccion en sitio propio</t>
+          <t>Fondo MiVivienda: construcción en sitio propio</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>FCR/ONP 2024: Banco de Materiales en liquidacion</t>
+          <t>FCR/ONP 2024: Banco de Materiales en liquidación</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Guia gob.pe: Plataforma de Interoperabilidad del Estado</t>
+          <t>Guía gob.pe: Plataforma de Interoperabilidad del Estado</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Datos Abiertos: resoluciones de licencias de edificacion MML</t>
+          <t>Datos Abiertos: resoluciones de licencias de edificación MML</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -4523,12 +4523,12 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Saneamiento fisico-legal y titularidad</t>
+          <t>Saneamiento físico-legal y titularidad</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Convertir la posesion o el contrato en propiedad inscrita en SUNARP.</t>
+          <t>Convertir la posesión o el contrato en propiedad inscrita en SUNARP.</t>
         </is>
       </c>
       <c r="E2" s="6" t="b">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Parametros urbanisticos, factibilidades y anteproyecto: definen que y cuanto se puede construir.</t>
+          <t>Parámetros urbanísticos, factibilidades y anteproyecto: definen qué y cuánto se puede construir.</t>
         </is>
       </c>
       <c r="E3" s="6" t="b">
@@ -4569,12 +4569,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Regularizacion de lo construido</t>
+          <t>Regularización de lo construido</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Solo si ya existe construccion sin licencia o sin declarar.</t>
+          <t>Solo si ya existe construcción sin licencia o sin declarar.</t>
         </is>
       </c>
       <c r="E4" s="6" t="b">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Solo si el predio esta en zona especial (Pantanos de Villa, ANP, zona monumental) o el proyecto lo exige.</t>
+          <t>Solo si el predio está en zona especial (Pantanos de Villa, ANP, zona monumental) o el proyecto lo exige.</t>
         </is>
       </c>
       <c r="E5" s="6" t="b">
@@ -4615,12 +4615,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion</t>
+          <t>Licencia de edificación</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Modalidad A, B, C o D segun tamano y uso.</t>
+          <t>Modalidad A, B, C o D según tamaño y uso.</t>
         </is>
       </c>
       <c r="E6" s="6" t="b">
@@ -4638,12 +4638,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Inicio y ejecucion de obra</t>
+          <t>Inicio y ejecución de obra</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Comunicacion de inicio, verificaciones tecnicas, seguros y obligaciones laborales.</t>
+          <t>Comunicación de inicio, verificaciones técnicas, seguros y obligaciones laborales.</t>
         </is>
       </c>
       <c r="E7" s="6" t="b">
@@ -4661,12 +4661,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra, declaratoria e inscripcion</t>
+          <t>Conformidad de obra, declaratoria e inscripción</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Cierre legal: conformidad municipal, inscripcion en SUNARP y actualizacion predial.</t>
+          <t>Cierre legal: conformidad municipal, inscripción en SUNARP y actualización predial.</t>
         </is>
       </c>
       <c r="E8" s="6" t="b">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Verifica titularidad, cargas y gravamenes antes de comprar o iniciar.</t>
+          <t>Verifica titularidad, cargas y gravámenes antes de comprar o iniciar.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -4840,7 +4840,7 @@
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Segun SUNARP</t>
+          <t>Según SUNARP</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Copia de la partida; la licencia exige antiguedad maxima de 30 dias.</t>
+          <t>Copia de la partida; la licencia exige antigüedad máxima de 30 días.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -4925,7 +4925,7 @@
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Inmediata en linea</t>
+          <t>Inmediata en línea</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -4937,7 +4937,7 @@
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>Publicidad registral en linea: S/ 5 por asiento/pagina</t>
+          <t>Publicidad registral en línea: S/ 5 por asiento/página</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Escritura publica de compraventa</t>
+          <t>Escritura pública de compraventa</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>El notario eleva la minuta a escritura publica y la presenta a SUNARP por SID-Sunarp.</t>
+          <t>El notario eleva la minuta a escritura pública y la presenta a SUNARP por SID-Sunarp.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -5010,7 +5010,7 @@
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Segun notaria</t>
+          <t>Según notaría</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de compraventa</t>
+          <t>Inscripción de compraventa</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Calificacion registral e inscripcion de la transferencia.</t>
+          <t>Calificación registral e inscripción de la transferencia.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -5109,7 +5109,7 @@
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Derecho de calificacion; mas derecho de inscripcion segun valor (usar Calculadora Registral)</t>
+          <t>Derecho de calificación; más derecho de inscripción según valor (usar Calculadora Registral)</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
@@ -5246,7 +5246,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Formalizacion de la propiedad (COFOPRI)</t>
+          <t>Formalización de la propiedad (COFOPRI)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Titulo gratuito para posesiones informales: terreno estatal ocupado hasta el 31-12-2021; privado con posesion pacifica de mas de 10 anos.</t>
+          <t>Título gratuito para posesiones informales: terreno estatal ocupado hasta el 31-12-2021; privado con posesión pacífica de más de 10 años.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -5267,7 +5267,7 @@
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Proceso por campanas</t>
+          <t>Proceso por campañas</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Prescripcion adquisitiva de dominio</t>
+          <t>Prescripción adquisitiva de dominio</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Via notarial o judicial para quien posee como propietario por mas de 10 anos.</t>
+          <t>Vía notarial o judicial para quien posee como propietario por más de 10 años.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -5350,7 +5350,7 @@
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Meses; varia por caso</t>
+          <t>Meses; varía por caso</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Sucesion intestada</t>
+          <t>Sucesión intestada</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Declara herederos cuando el titular fallecio sin testamento; luego se inscribe en SUNARP.</t>
+          <t>Declara herederos cuando el titular falleció sin testamento; luego se inscribe en SUNARP.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Subdivision de lote</t>
+          <t>Subdivisión de lote</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Independizacion registral</t>
+          <t>Independización registral</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -5608,7 +5608,7 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>S/ 89-99 por unidad resultante + calificacion</t>
+          <t>S/ 89-99 por unidad resultante + calificación</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Parametros Urbanisticos y Edificatorios</t>
+          <t>Certificado de Parámetros Urbanísticos y Edificatorios</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Zonificacion, altura, retiros, area libre, densidad y estacionamientos del predio.</t>
+          <t>Zonificación, altura, retiros, área libre, densidad y estacionamientos del predio.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Zonificacion y Vias</t>
+          <t>Certificado de Zonificación y Vías</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Uso de suelo y seccion vial (principalmente habilitaciones urbanas).</t>
+          <t>Uso de suelo y sección vial (principalmente habilitaciones urbanas).</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -5829,7 +5829,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Factibilidad de agua y desague</t>
+          <t>Factibilidad de agua y desagüe</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -5912,7 +5912,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Factibilidad electrica</t>
+          <t>Factibilidad eléctrica</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -5993,7 +5993,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Asignacion / certificado de numeracion</t>
+          <t>Asignación / certificado de numeración</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Numeracion municipal del predio.</t>
+          <t>Numeración municipal del predio.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Revision del diseno antes del expediente completo; reduce observaciones.</t>
+          <t>Revisión del diseño antes del expediente completo; reduce observaciones.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Declaratoria de fabrica por regularizacion (Ley 27157)</t>
+          <t>Declaratoria de fábrica por regularización (Ley 27157)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -6183,7 +6183,7 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>S/ 41-50 fijo + 3/1000 del valor de la construccion</t>
+          <t>S/ 41-50 fijo + 3/1000 del valor de la construcción</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion en via de regularizacion</t>
+          <t>Licencia de edificación en vía de regularización</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Beneficio municipal de regularizacion (por ordenanza temporal)</t>
+          <t>Beneficio municipal de regularización (por ordenanza temporal)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Para obras posteriores al 17-09-2018 solo si el distrito tiene una ordenanza vigente. Ej.: Surco Ord. 682-MSS (obras 18-09-2018 a 31-12-2022), vencio el 17-07-2025.</t>
+          <t>Para obras posteriores al 17-09-2018 solo si el distrito tiene una ordenanza vigente. Ej.: Surco Ord. 682-MSS (obras 18-09-2018 a 31-12-2022), venció el 17-07-2025.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -6350,7 +6350,7 @@
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>Segun ordenanza</t>
+          <t>Según ordenanza</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Opinion ambiental PROHVILLA</t>
+          <t>Opinión ambiental PROHVILLA</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -6423,7 +6423,7 @@
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Suele demorar; en el caso real de referencia fue la etapa mas larga</t>
+          <t>Suele demorar; en el caso real de referencia fue la etapa más larga</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -6435,7 +6435,7 @@
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>Tasa segun TUPA MML/PROHVILLA</t>
+          <t>Tasa según TUPA MML/PROHVILLA</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Compatibilidad y opinion tecnica previa vinculante SERNANP</t>
+          <t>Compatibilidad y opinión técnica previa vinculante SERNANP</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Actividades en areas naturales protegidas de administracion nacional o su zona de amortiguamiento.</t>
+          <t>Actividades en áreas naturales protegidas de administración nacional o su zona de amortiguamiento.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -6516,7 +6516,7 @@
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Segun SERNANP</t>
+          <t>Según SERNANP</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Autorizacion del Ministerio de Cultura</t>
+          <t>Autorización del Ministerio de Cultura</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -6730,13 +6730,13 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Certificacion ambiental</t>
+          <t>Certificación ambiental</t>
         </is>
       </c>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Segun tipo y escala del proyecto (C/D).</t>
+          <t>Según tipo y escala del proyecto (C/D).</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad A (aprobacion automatica)</t>
+          <t>Licencia de edificación - Modalidad A (aprobación automática)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Vivienda unifamiliar nueva hasta 120 m2; ampliacion hasta 200 m2 totales; remodelacion sin cambio estructural; cercos de mas de 20 m; demolicion hasta 3 pisos; obras menores.</t>
+          <t>Vivienda unifamiliar nueva hasta 120 m²; ampliación hasta 200 m² totales; remodelación sin cambio estructural; cercos de más de 20 m; demolición hasta 3 pisos; obras menores.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>Licencia al ingreso; verificacion administrativa en 10 dias habiles</t>
+          <t>Licencia al ingreso; verificación administrativa en 10 días hábiles</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad B (evaluacion municipal)</t>
+          <t>Licencia de edificación - Modalidad B (evaluación municipal)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -6904,7 +6904,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Vivienda hasta 5 pisos y hasta 3,000 m2; ampliaciones o remodelaciones con cambio estructural; demolicion parcial.</t>
+          <t>Vivienda hasta 5 pisos y hasta 3,000 m²; ampliaciones o remodelaciones con cambio estructural; demolición parcial.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>15 dias habiles (Pueblo Libre, La Molina)</t>
+          <t>15 días hábiles (Pueblo Libre, La Molina)</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad B (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad B (revisores urbanos)</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -6991,7 +6991,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Mismo alcance que B; el proyecto llega con informe tecnico favorable de revisores urbanos y la municipalidad cobra una tasa menor.</t>
+          <t>Mismo alcance que B; el proyecto llega con informe técnico favorable de revisores urbanos y la municipalidad cobra una tasa menor.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad C (comision tecnica)</t>
+          <t>Licencia de edificación - Modalidad C (comisión técnica)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Vivienda multifamiliar de mas de 5 pisos o mas de 3,000 m2; usos distintos a vivienda; uso mixto; patrimonio cultural; comercio hasta 30,000 m2; mercados hasta 15,000 m2.</t>
+          <t>Vivienda multifamiliar de más de 5 pisos o más de 3,000 m²; usos distintos a vivienda; uso mixto; patrimonio cultural; comercio hasta 30,000 m²; mercados hasta 15,000 m².</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Hasta 25 dias habiles de evaluacion de comision (La Molina, flujo anterior)</t>
+          <t>Hasta 25 días hábiles de evaluación de comisión (La Molina, flujo anterior)</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad C (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad C (revisores urbanos)</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad D (comision tecnica)</t>
+          <t>Licencia de edificación - Modalidad D (comisión técnica)</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Industria; comercio de mas de 30,000 m2; mercados de mas de 15,000 m2; educacion, salud, hospedaje.</t>
+          <t>Industria; comercio de más de 30,000 m²; mercados de más de 15,000 m²; educación, salud, hospedaje.</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Licencia de edificacion - Modalidad D (revisores urbanos)</t>
+          <t>Licencia de edificación - Modalidad D (revisores urbanos)</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Modificacion de proyecto (antes o despues de la licencia; sustancial o no sustancial)</t>
+          <t>Modificación de proyecto (antes o después de la licencia; sustancial o no sustancial)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -7479,7 +7479,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Prorroga de licencia (12 meses)</t>
+          <t>Prórroga de licencia (12 meses)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Unica prorroga; debe pedirse antes del vencimiento de los 36 meses.</t>
+          <t>Única prórroga; debe pedirse antes del vencimiento de los 36 meses.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Revalidacion de licencia</t>
+          <t>Revalidación de licencia</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Cuando la licencia ya vencio.</t>
+          <t>Cuando la licencia ya venció.</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Comunicacion de inicio de obra (Anexo H)</t>
+          <t>Comunicación de inicio de obra (Anexo H)</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Aviso formal antes de iniciar, con cronograma de verificaciones tecnicas.</t>
+          <t>Aviso formal antes de iniciar, con cronograma de verificaciones técnicas.</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -7678,7 +7678,7 @@
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="inlineStr">
         <is>
-          <t>Segun TUPA; en varios distritos sin costo</t>
+          <t>Según TUPA; en varios distritos sin costo</t>
         </is>
       </c>
       <c r="M36" s="6" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Verificaciones tecnicas durante la obra</t>
+          <t>Verificaciones técnicas durante la obra</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -7740,7 +7740,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Visitas en hitos (cimentacion, albanileria, techos). Desvios respecto a planos pueden derivar en paralizacion.</t>
+          <t>Visitas en hitos (cimentación, albañilería, techos). Desvíos respecto a planos pueden derivar en paralización.</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -7763,7 +7763,7 @@
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="inlineStr">
         <is>
-          <t>Segun TUPA</t>
+          <t>Según TUPA</t>
         </is>
       </c>
       <c r="M37" s="6" t="inlineStr">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Contratar poliza CAR o de responsabilidad civil</t>
+          <t>Contratar póliza CAR o de responsabilidad civil</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -7825,7 +7825,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Cobertura por danos a terceros durante toda la obra (C y D, y segun reglamento).</t>
+          <t>Cobertura por daños a terceros durante toda la obra (C y D, y según reglamento).</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de la obra en RENOCC</t>
+          <t>Inscripción de la obra en RENOCC</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Obligatoria para obras de construccion civil de mas de 50 UIT (S/ 275,000 en 2026).</t>
+          <t>Obligatoria para obras de construcción civil de más de 50 UIT (S/ 275,000 en 2026).</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -7925,7 +7925,7 @@
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="6" t="inlineStr">
         <is>
-          <t>Segun MTPE</t>
+          <t>Según MTPE</t>
         </is>
       </c>
       <c r="M39" s="6" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Registro de trabajadores de construccion civil (RETCC)</t>
+          <t>Registro de trabajadores de construcción civil (RETCC)</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Trabajadores del regimen de construccion civil deben estar registrados.</t>
+          <t>Trabajadores del régimen de construcción civil deben estar registrados.</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -8006,7 +8006,7 @@
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="inlineStr">
         <is>
-          <t>Segun MTPE</t>
+          <t>Según MTPE</t>
         </is>
       </c>
       <c r="M40" s="6" t="inlineStr">
@@ -8068,7 +8068,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Obligatorio para actividades de riesgo, incluida construccion.</t>
+          <t>Obligatorio para actividades de riesgo, incluida construcción.</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -8149,7 +8149,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Aporte de los obreros de construccion civil, retenido por el empleador.</t>
+          <t>Aporte de los obreros de construcción civil, retenido por el empleador.</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -8172,7 +8172,7 @@
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>Porcentaje del jornal basico por confirmar</t>
+          <t>Porcentaje del jornal básico por confirmar</t>
         </is>
       </c>
       <c r="M42" s="6" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Contribucion sobre ingresos por obras de construccion. Confirmar si aplica a autoconstruccion familiar.</t>
+          <t>Contribución sobre ingresos por obras de construcción. Confirmar si aplica a autoconstrucción familiar.</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Cartel de obra con numero de licencia</t>
+          <t>Cartel de obra con número de licencia</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Visible durante toda la ejecucion.</t>
+          <t>Visible durante toda la ejecución.</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -8386,7 +8386,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra y declaratoria de edificacion sin variaciones</t>
+          <t>Conformidad de obra y declaratoria de edificación sin variaciones</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Conformidad de obra y declaratoria de edificacion con variaciones</t>
+          <t>Conformidad de obra y declaratoria de edificación con variaciones</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Predeclaratoria de edificacion</t>
+          <t>Predeclaratoria de edificación</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de la declaratoria de edificacion</t>
+          <t>Inscripción de la declaratoria de edificación</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -8738,7 +8738,7 @@
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Calificacion (~S/ 41-50) + 3/1000 del valor de la obra</t>
+          <t>Calificación (~S/ 41-50) + 3/1000 del valor de la obra</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Inscripcion de reglamento interno e independizacion de unidades</t>
+          <t>Inscripción de reglamento interno e independización de unidades</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Multifamiliares: cada departamento, estacionamiento o deposito con partida propia.</t>
+          <t>Multifamiliares: cada departamento, estacionamiento o depósito con partida propia.</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -8823,7 +8823,7 @@
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>S/ 89-99 por unidad + calificacion</t>
+          <t>S/ 89-99 por unidad + calificación</t>
         </is>
       </c>
       <c r="L50" s="6" t="n"/>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Actualizar declaracion jurada del impuesto predial</t>
+          <t>Actualizar declaración jurada del impuesto predial</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -9012,7 +9012,7 @@
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Identificacion.</t>
+          <t>Identificación.</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
@@ -9040,7 +9040,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Punto de partida cuando la propiedad no esta inscrita.</t>
+          <t>Punto de partida cuando la propiedad no está inscrita.</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -9057,7 +9057,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Escritura publica</t>
+          <t>Escritura pública</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -9096,7 +9096,7 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Muestra cargas, gravamenes y titularidad.</t>
+          <t>Muestra cargas, gravámenes y titularidad.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>La licencia exige una copia con antiguedad maxima de 30 dias.</t>
+          <t>La licencia exige una copia con antigüedad máxima de 30 días.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -9143,7 +9143,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Titulo de propiedad COFOPRI inscrito</t>
+          <t>Título de propiedad COFOPRI inscrito</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -9154,7 +9154,7 @@
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Resultado de la formalizacion.</t>
+          <t>Resultado de la formalización.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Sucesion intestada o testamento inscrito</t>
+          <t>Sucesión intestada o testamento inscrito</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -9182,7 +9182,7 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Necesario si el titular registral fallecio.</t>
+          <t>Necesario si el titular registral falleció.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -9212,7 +9212,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Si tramita un representante o persona juridica.</t>
+          <t>Si tramita un representante o persona jurídica.</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
@@ -9229,7 +9229,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Parametros Urbanisticos y Edificatorios</t>
+          <t>Certificado de Parámetros Urbanísticos y Edificatorios</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Certificado de Zonificacion y Vias</t>
+          <t>Certificado de Zonificación y Vías</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Certificado de factibilidad de agua y desague</t>
+          <t>Certificado de factibilidad de agua y desagüe</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -9302,7 +9302,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Vigencia 36 meses segun Pueblo Libre.</t>
+          <t>Vigencia 36 meses según Pueblo Libre.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Certificado de factibilidad electrica</t>
+          <t>Certificado de factibilidad eléctrica</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Luz del Sur o Enel segun zona. Vigencia por confirmar.</t>
+          <t>Luz del Sur o Enel según zona. Vigencia por confirmar.</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Formulario Unico de Edificaciones (FUE)</t>
+          <t>Formulario Único de Edificaciones (FUE)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Anexos del FUE (A: condominos, B, D: autoliquidacion, H: inicio de obra)</t>
+          <t>Anexos del FUE (A: condóminos, B, D: autoliquidación, H: inicio de obra)</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -9384,7 +9384,7 @@
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Anexo H = comunicacion de inicio de obra.</t>
+          <t>Anexo H = comunicación de inicio de obra.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Plano de ubicacion y localizacion</t>
+          <t>Plano de ubicación y localización</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
@@ -9497,7 +9497,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Planos de instalaciones electricas</t>
+          <t>Planos de instalaciones eléctricas</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
@@ -9521,14 +9521,14 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Estudio de Mecanica de Suelos (EMS)</t>
+          <t>Estudio de Mecánica de Suelos (EMS)</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Surco: obligatorio desde 4 pisos o mas de 500 m2 en primer piso.</t>
+          <t>Surco: obligatorio desde 4 pisos o más de 500 m² en primer piso.</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -9552,7 +9552,7 @@
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Excavaciones de mas de 2 m.</t>
+          <t>Excavaciones de más de 2 m.</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -9569,14 +9569,14 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Planos de seguridad y evacuacion</t>
+          <t>Planos de seguridad y evacuación</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Edificios de mas de 5 pisos y usos con afluencia de publico.</t>
+          <t>Edificios de más de 5 pisos y usos con afluencia de público.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Poliza CAR o de responsabilidad civil</t>
+          <t>Póliza CAR o de responsabilidad civil</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -9697,14 +9697,14 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Certificacion ambiental</t>
+          <t>Certificación ambiental</t>
         </is>
       </c>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Segun tipo de proyecto (C/D).</t>
+          <t>Según tipo de proyecto (C/D).</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -9721,7 +9721,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Opinion ambiental de PROHVILLA</t>
+          <t>Opinión ambiental de PROHVILLA</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Compatibilidad / opinion tecnica previa vinculante SERNANP</t>
+          <t>Compatibilidad / opinión técnica previa vinculante SERNANP</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Autorizacion del Ministerio de Cultura</t>
+          <t>Autorización del Ministerio de Cultura</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -9835,7 +9835,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Resolucion de licencia de edificacion</t>
+          <t>Resolución de licencia de edificación</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -9876,7 +9876,7 @@
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Declaratoria de fabrica por regularizacion.</t>
+          <t>Declaratoria de fábrica por regularización.</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
@@ -9893,7 +9893,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Informe tecnico del verificador responsable</t>
+          <t>Informe técnico del verificador responsable</t>
         </is>
       </c>
       <c r="C35" s="6" t="n"/>
@@ -9945,7 +9945,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Cronograma de visitas de verificacion tecnica</t>
+          <t>Cronograma de visitas de verificación técnica</t>
         </is>
       </c>
       <c r="C37" s="6" t="n"/>
@@ -9969,7 +9969,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Poliza SCTR (salud y pension)</t>
+          <t>Póliza SCTR (salud y pensión)</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
@@ -9980,7 +9980,7 @@
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Obligatoria para trabajadores de construccion civil.</t>
+          <t>Obligatoria para trabajadores de construcción civil.</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Constancia de inscripcion de obra en RENOCC</t>
+          <t>Constancia de inscripción de obra en RENOCC</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
@@ -10008,7 +10008,7 @@
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Obras de mas de 50 UIT.</t>
+          <t>Obras de más de 50 UIT.</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -10049,7 +10049,7 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Resolucion de conformidad de obra y declaratoria de edificacion</t>
+          <t>Resolución de conformidad de obra y declaratoria de edificación</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Autoriza la inscripcion registral.</t>
+          <t>Autoriza la inscripción registral.</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -10084,7 +10084,7 @@
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Multifamiliares / propiedad exclusiva y comun.</t>
+          <t>Multifamiliares / propiedad exclusiva y común.</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -10101,7 +10101,7 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Declaracion jurada de autoavaluo actualizada</t>
+          <t>Declaración jurada de autoavalúo actualizada</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Superintendencia Nacional de los Registros Publicos</t>
+          <t>Superintendencia Nacional de los Registros Públicos</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>SID-Sunarp (notarios), Publicidad Registral en Linea, Siguelo, Alerta Registral</t>
+          <t>SID-Sunarp (notarios), Publicidad Registral en Línea, Síguelo, Alerta Registral</t>
         </is>
       </c>
     </row>
@@ -10227,7 +10227,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Notaria publica</t>
+          <t>Notaría pública</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -10248,7 +10248,7 @@
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Presencial; presenta a SUNARP via SID-Sunarp</t>
+          <t>Presencial; presenta a SUNARP vía SID-Sunarp</t>
         </is>
       </c>
     </row>
@@ -10260,7 +10260,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Organismo de Formalizacion de la Propiedad Informal</t>
+          <t>Organismo de Formalización de la Propiedad Informal</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -10285,7 +10285,7 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Campanas y oficinas</t>
+          <t>Campañas y oficinas</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Mesa de partes electronica</t>
+          <t>Mesa de partes electrónica</t>
         </is>
       </c>
     </row>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Municipalidad distrital (segun ubicacion del predio)</t>
+          <t>Municipalidad distrital (según ubicación del predio)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -10355,7 +10355,7 @@
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Varia por distrito: ver distritos.json</t>
+          <t>Varía por distrito: ver distritos.json</t>
         </is>
       </c>
     </row>
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Servicio de Administracion Tributaria de Lima</t>
+          <t>Servicio de Administración Tributaria de Lima</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -10466,7 +10466,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Tramite en gob.pe</t>
+          <t>Trámite en gob.pe</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Servicio Nacional de Areas Naturales Protegidas</t>
+          <t>Servicio Nacional de Áreas Naturales Protegidas</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -10503,7 +10503,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Modulo de Compatibilidad en linea</t>
+          <t>Módulo de Compatibilidad en línea</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de Vivienda, Construccion y Saneamiento</t>
+          <t>Ministerio de Vivienda, Construcción y Saneamiento</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -10577,7 +10577,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Plataforma de tramites digitales</t>
+          <t>Plataforma de trámites digitales</t>
         </is>
       </c>
     </row>
@@ -10614,7 +10614,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Postulacion en linea, 0800-12-200</t>
+          <t>Postulación en línea, 0800-12-200</t>
         </is>
       </c>
     </row>
@@ -10626,7 +10626,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Ministerio de Trabajo y Promocion del Empleo</t>
+          <t>Ministerio de Trabajo y Promoción del Empleo</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -10651,7 +10651,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Registros de construccion civil en linea</t>
+          <t>Registros de construcción civil en línea</t>
         </is>
       </c>
     </row>
@@ -10725,7 +10725,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Atencion virtual; atiende Lima Sur y Este</t>
+          <t>Atención virtual; atiende Lima Sur y Este</t>
         </is>
       </c>
     </row>
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Enel Distribucion Peru</t>
+          <t>Enel Distribución Perú</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -10762,7 +10762,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Atencion virtual; atiende Lima Norte y Oeste</t>
+          <t>Atención virtual; atiende Lima Norte y Oeste</t>
         </is>
       </c>
     </row>
@@ -10774,7 +10774,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Colegio de Arquitectos / Colegio de Ingenieros del Peru</t>
+          <t>Colegio de Arquitectos / Colegio de Ingenieros del Perú</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -10795,7 +10795,7 @@
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Delegados en comisiones tecnicas; habilidad profesional</t>
+          <t>Delegados en comisiones técnicas; habilidad profesional</t>
         </is>
       </c>
     </row>
@@ -10828,7 +10828,7 @@
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Alternativa a la municipalidad/comision en B, C y D</t>
+          <t>Alternativa a la municipalidad/comisión en B, C y D</t>
         </is>
       </c>
     </row>
@@ -10840,7 +10840,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Compania de seguros</t>
+          <t>Compañía de seguros</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -10861,7 +10861,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Poliza CAR / responsabilidad civil / SCTR</t>
+          <t>Póliza CAR / responsabilidad civil / SCTR</t>
         </is>
       </c>
     </row>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Servicio Nacional de Capacitacion para la Industria de la Construccion</t>
+          <t>Servicio Nacional de Capacitación para la Industria de la Construcción</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Declaracion y pago</t>
+          <t>Declaración y pago</t>
         </is>
       </c>
     </row>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Fondo de Vivienda del Trabajador de Construccion Civil</t>
+          <t>Fondo de Vivienda del Trabajador de Construcción Civil</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Retencion por el empleador</t>
+          <t>Retención por el empleador</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Participan en comision tecnica</t>
+          <t>Participan en comisión técnica</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>El PDF publicado no expone montos legibles de edificacion; confirmar TUPA vigente y su adecuacion al D.S. 146-2023-PCM.</t>
+          <t>El PDF publicado no expone montos legibles de edificación; confirmar TUPA vigente y su adecuación al D.S. 146-2023-PCM.</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -11158,7 +11158,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>TUPA publicado el 27-09-2024 (220 procedimientos). Montos de licencias tomados de la version 2022: confirmar.</t>
+          <t>TUPA publicado el 27-09-2024 (220 procedimientos). Montos de licencias tomados de la versión 2022: confirmar.</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -11212,7 +11212,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>TUPA 2025 ratificado por la MML; 123 procedimientos de HU y edificacion adecuados al D.S. 146-2023-PCM (vigente desde 22-06-2024). Montos por extraer del anexo.</t>
+          <t>TUPA 2025 ratificado por la MML; 123 procedimientos de HU y edificación adecuados al D.S. 146-2023-PCM (vigente desde 22-06-2024). Montos por extraer del anexo.</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Distrito de referencia: unico con tasas completas extraidas (TUPA 2025, UIT 5,350).</t>
+          <t>Distrito de referencia: único con tasas completas extraídas (TUPA 2025, UIT 5,350).</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -12876,7 +12876,7 @@
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>Monto atipicamente bajo en la extraccion: confirmar</t>
+          <t>Monto atípicamente bajo en la extracción: confirmar</t>
         </is>
       </c>
     </row>
@@ -13204,7 +13204,7 @@
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>Rango 2022: S/ 56.10 a 122.20 segun submodalidad</t>
+          <t>Rango 2022: S/ 56.10 a 122.20 según submodalidad</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13480,7 @@
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13524,7 +13524,7 @@
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13568,7 +13568,7 @@
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13612,7 +13612,7 @@
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13656,7 +13656,7 @@
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13700,7 +13700,7 @@
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13744,7 +13744,7 @@
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13788,7 +13788,7 @@
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13832,7 +13832,7 @@
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13876,7 +13876,7 @@
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13920,7 +13920,7 @@
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -13964,7 +13964,7 @@
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14008,7 +14008,7 @@
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14052,7 +14052,7 @@
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14140,7 +14140,7 @@
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14184,7 +14184,7 @@
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14228,7 +14228,7 @@
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>Codigo del TUPA 2021; monto por extraer</t>
+          <t>Código del TUPA 2021; monto por extraer</t>
         </is>
       </c>
     </row>
@@ -14595,7 +14595,7 @@
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>{"alturas_pisos": "2 a 4 (zonas residenciales RDMB, RDB, RDM)", "area_libre_pct": "30 a 60", "retiro_frontal_m": "5 a 25", "otros": "Arborizacion obligatoria; restriccion de subdivisiones; ZHR max. 2 pisos; IE max. 1 piso"}</t>
+          <t>{"alturas_pisos": "2 a 4 (zonas residenciales RDMB, RDB, RDM)", "area_libre_pct": "30 a 60", "retiro_frontal_m": "5 a 25", "otros": "Arborización obligatoria; restricción de subdivisiones; ZHR max. 2 pisos; IE max. 1 piso"}</t>
         </is>
       </c>
       <c r="I2" s="6" t="n"/>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Area Natural Protegida nacional o su zona de amortiguamiento</t>
+          <t>Área Natural Protegida nacional o su zona de amortiguamiento</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -14803,7 +14803,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Techo Propio - Construccion en Sitio Propio</t>
+          <t>Techo Propio - Construcción en Sitio Propio</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>["Ingreso familiar mensual hasta S/ 2,706", "Ahorro minimo S/ 2,475", "Terreno o aires inscritos en SUNARP", "No tener otra propiedad ni beneficio previo", "Grupo familiar constituido"]</t>
+          <t>["Ingreso familiar mensual hasta S/ 2,706", "Ahorro mínimo S/ 2,475", "Terreno o aires inscritos en SUNARP", "No tener otra propiedad ni beneficio previo", "Grupo familiar constituido"]</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -14851,7 +14851,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Techo Propio - Adquisicion de Vivienda Nueva</t>
+          <t>Techo Propio - Adquisición de Vivienda Nueva</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Segun convocatoria</t>
+          <t>Según convocatoria</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Creditos MiVivienda y productos de construccion</t>
+          <t>Créditos MiVivienda y productos de construcción</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Credito hipotecario via bancos y cajas</t>
+          <t>Crédito hipotecario vía bancos y cajas</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Formalizacion gratuita COFOPRI</t>
+          <t>Formalización gratuita COFOPRI</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -14960,12 +14960,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Titulo de propiedad gratuito inscrito</t>
+          <t>Título de propiedad gratuito inscrito</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>["Terreno estatal ocupado hasta 31-12-2021 o privado con posesion de mas de 10 anos"]</t>
+          <t>["Terreno estatal ocupado hasta 31-12-2021 o privado con posesión de más de 10 años"]</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>En liquidacion: no otorga creditos nuevos</t>
+          <t>En liquidación: no otorga créditos nuevos</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
data: URL de F-DATOS-CONF-MML con www (sin www no resuelve)
La vigilancia (issue #19) la reportó sin respuesta: datosabiertos.gob.pe sin
www no resuelve. Con www responde 200 y es el mismo dataset ("Conformidad de
Obra y Declaratoria de Edificación - MML"). Se actualiza fecha_consulta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ruta-obra.xlsx
+++ b/data/ruta-obra.xlsx
@@ -4449,7 +4449,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>https://datosabiertos.gob.pe/dataset/conformidad-de-obra-y-declaratoria-de-edificaci%C3%B3n-municipalidad-metropolitana-de-lima-0</t>
+          <t>https://www.datosabiertos.gob.pe/dataset/conformidad-de-obra-y-declaratoria-de-edificaci%C3%B3n-municipalidad-metropolitana-de-lima-0</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: URL de F-DATOS-CONF-MML con www (sin www no resuelve) (#21)
La vigilancia (issue #19) la reportó sin respuesta: datosabiertos.gob.pe sin
www no resuelve. Con www responde 200 y es el mismo dataset ("Conformidad de
Obra y Declaratoria de Edificación - MML"). Se actualiza fecha_consulta.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ruta-obra.xlsx
+++ b/data/ruta-obra.xlsx
@@ -4449,7 +4449,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>https://datosabiertos.gob.pe/dataset/conformidad-de-obra-y-declaratoria-de-edificaci%C3%B3n-municipalidad-metropolitana-de-lima-0</t>
+          <t>https://www.datosabiertos.gob.pe/dataset/conformidad-de-obra-y-declaratoria-de-edificaci%C3%B3n-municipalidad-metropolitana-de-lima-0</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>